<commit_message>
edits to some plot labels
</commit_message>
<xml_diff>
--- a/B8 Unit Cell - k_inf/modr-fuel-ratio.xlsx
+++ b/B8 Unit Cell - k_inf/modr-fuel-ratio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MCNP\haigerloch-modr-fuel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MCNP\b8pile\B8 Unit Cell - k_inf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479710F9-89E7-4635-8E7A-9D5340A6300D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365CB527-59C6-4275-824D-C97E18E018E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1200,6 +1200,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1207,7 +1208,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1776,7 +1776,7 @@
                     <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                     <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
                   </a:rPr>
-                  <a:t>inf</a:t>
+                  <a:t>∞</a:t>
                 </a:r>
                 <a:r>
                   <a:rPr lang="en-US">
@@ -1867,6 +1867,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1874,7 +1875,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:noFill/>

</xml_diff>